<commit_message>
V8-003 Final Release 보고서 생성 안정화
</commit_message>
<xml_diff>
--- a/output/2026-05/판매수수료_전년대비보고서.xlsx
+++ b/output/2026-05/판매수수료_전년대비보고서.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="표1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구분" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피벗값_구분" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피벗값_매장명(동일)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피벗값_매장명(동일) 값_영업이익순" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피벗값_매장명 (폐점)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피벗값_매장명 (행사)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피벗값_매장명 (신규)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="표1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="구분" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="피벗값_구분" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="피벗값_매장명(동일)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="피벗값_매장명(동일) 값_영업이익순" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="피벗값_매장명 (폐점)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="피벗값_매장명 (행사)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="피벗값_매장명 (신규)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'표1'!$A$1:$N$638</definedName>
@@ -284,14 +284,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -315,7 +315,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -339,7 +339,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -379,8 +379,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -406,7 +406,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -421,9 +421,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>